<commit_message>
def: repair stale bindings - TargetSample -> DesignSample (sampleMatrix, samplerInsertionMethod, descriptions incl. sampleType), triaxType drops diggs_geo twins, geosyntheticReinforcementType also binds Geosynthetic/reinforcementType
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/geosyntheticReinforcementType.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/geosyntheticReinforcementType.xlsx
@@ -985,7 +985,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes for a geosynthetic reinforcement layer's product form - geogrid or geotextile, and the axiality of a geogrid. Distinct from diggs:reinforcementType on diggs:ReinforcementType (steel cage arrangement) despite the shared element name - a different object, a different vocabulary. Used for the value of diggs:DesignGeosyntheticLayerType/diggs:reinforcementType.</t>
+          <t>Codes for a geosynthetic reinforcement layer's product form - geogrid or geotextile, and the axiality of a geogrid. Distinct from diggs:reinforcementType on diggs:ReinforcementType (steel cage arrangement) despite the shared element name - a different object, a different vocabulary. Used for the value of diggs:DesignGeosyntheticLayerType/reinforcementType and diggs:GeosyntheticType/reinforcementType.</t>
         </is>
       </c>
     </row>
@@ -1671,28 +1671,64 @@
         <f>IF(ISNA(VLOOKUP(B6,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B6" s="2" t="n"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>geogrid_uniaxial</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>//diggs:Geosynthetic/diggs:reinforcementType</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
         <f>IF(ISNA(VLOOKUP(B7,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B7" s="2" t="n"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>geogrid_biaxial</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>//diggs:Geosynthetic/diggs:reinforcementType</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
         <f>IF(ISNA(VLOOKUP(B8,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B8" s="2" t="n"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>geogrid_triaxial</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>//diggs:Geosynthetic/diggs:reinforcementType</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
         <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B9" s="2" t="n"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>geotextile_woven</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>//diggs:Geosynthetic/diggs:reinforcementType</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10">

</xml_diff>